<commit_message>
Refresh machine-readable tables and release manifest
</commit_message>
<xml_diff>
--- a/journal_outputs/machine_readable_tables.xlsx
+++ b/journal_outputs/machine_readable_tables.xlsx
@@ -26,6 +26,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="S14_TARGET_SUPPORT_SENSITIVITY" sheetId="17" state="visible" r:id="rId17"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="S15_NMI_NCS_RECORD_OVERLAP" sheetId="18" state="visible" r:id="rId18"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="S16_INDEPENDENT_SOURCE_RELEASE" sheetId="19" state="visible" r:id="rId19"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="S17_TEMPORAL_MODEL_SPECS" sheetId="20" state="visible" r:id="rId20"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'1_EXTERNAL_SOURCE_DESIGN'!$A$1:$Y$3</definedName>
@@ -2036,7 +2037,7 @@
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>Database versions and hashes are recorded; the final public archive DOI and restricted-source access route remain pending.</t>
+          <t>Database versions and hashes are recorded; the public repository is https://github.com/peizhang2235/representation-aware-protein-ligand-benchmark; a persistent archive DOI will be added at latest before the first revision, and restricted-source access remains provider-controlled.</t>
         </is>
       </c>
     </row>
@@ -2068,7 +2069,7 @@
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>Versioned scripts are packaged; a permanent repository DOI has not yet been minted.</t>
+          <t>Versioned scripts are publicly available at https://github.com/peizhang2235/representation-aware-protein-ligand-benchmark; a permanent repository DOI will be added at latest before the first revision.</t>
         </is>
       </c>
     </row>
@@ -3282,7 +3283,7 @@
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>JBD_v1_7</t>
+          <t>study_v1_7</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
@@ -3314,7 +3315,7 @@
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>The JBD manuscript remains a measurement-validity and external-generalization study.</t>
+          <t>The present manuscript remains a measurement-validity and external-generalization study.</t>
         </is>
       </c>
     </row>
@@ -3853,7 +3854,7 @@
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>Retrospective outcome-blind adaptation, not original prospective registry</t>
+          <t>Retrospective outcome-unexposed, structure-adapted adaptation, not original prospective registry</t>
         </is>
       </c>
     </row>
@@ -37836,7 +37837,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>independent_external_validation_already_in_JBD</t>
+          <t>independent_external_validation_already_in_JCHEMINF</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -37958,7 +37959,7 @@
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>GtoPdb ODbL database and CC BY-SA 4.0 contents; raw release not copied into JBD archive</t>
+          <t>GtoPdb ODbL database and CC BY-SA 4.0 contents; raw release not copied into public archive</t>
         </is>
       </c>
       <c r="M3" t="inlineStr">
@@ -37980,7 +37981,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>primary_JBD_external_source</t>
+          <t>primary_JCHEMINF_external_source</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -38035,7 +38036,7 @@
       </c>
       <c r="M4" t="inlineStr">
         <is>
-          <t>Current ChEMBL release used for JBD retrospective external evaluation.</t>
+          <t>Current ChEMBL release used for JCHEMINF retrospective external evaluation.</t>
         </is>
       </c>
       <c r="N4" t="inlineStr">
@@ -38052,7 +38053,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>JBD_temporal_source</t>
+          <t>JCHEMINF_temporal_source</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -41152,6 +41153,212 @@
     </row>
   </sheetData>
   <autoFilter ref="A1:J77"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet20.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F6"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>model</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>representation</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>architecture</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>training_cohort</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>prediction_interval_rule</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>frozen_state</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Frozen development median</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Exact development pKd labels</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>No learned architecture</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Development exact-label cohort</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>Prediction = development median; q90 = finite-sample 90th percentile of absolute development residuals</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>Frozen reference</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Morgan similarity</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>2048-bit Morgan fingerprint, radius 2</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Top-five Tanimoto local predictor; weights max(similarity, 1e-6)^4</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Development exact-label cohort</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>Weighted top-five prediction; q90 from frozen local-similarity calibration artifact</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>Frozen similarity artifact; no temporal outcome</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Additive HGB</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Ligand and protein feature fusion</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Histogram-gradient boosting with additive ligand/protein feature fusion</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Pre-2018 development cohort</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>Frozen HGB prediction; q90 = artifact.conformal_q90</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>Fixed model and calibration artifact</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Ligand MPNN + frozen ESM-2</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Ligand graph/message passing plus 320-dimensional ESM-2 protein embedding</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Ligand message-passing neural network combined with frozen ESM-2 features</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Pre-2018 development cohort</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Frozen graph-bundle prediction; q90 = graph bundle conformal_q90</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>Fixed model bundle and embedding revision</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>SMILES-protein cross-attention</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>SMILES/protein token representations</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Token model with SMILES-protein cross-attention; dimensions, heads, maximum lengths, and seed fixed in bundle</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Pre-2018 development cohort</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>Frozen joint-bundle prediction; q90 = joint bundle conformal_q90</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>Fixed model bundle; no temporal refit</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Align machine-readable tables with final supplement
</commit_message>
<xml_diff>
--- a/journal_outputs/machine_readable_tables.xlsx
+++ b/journal_outputs/machine_readable_tables.xlsx
@@ -2032,7 +2032,7 @@
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>Table 1; Table S6; release_materials/DATA_AND_CODE_AVAILABILITY_DRAFT.md</t>
+          <t>Table 1; Table S6; README.md and release_metadata/DATA_RIGHTS_MATRIX.md</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
@@ -2064,7 +2064,7 @@
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>scripts/; qc/; release_materials/REPRODUCIBILITY_COMMANDS.md</t>
+          <t>retrospective_v1_7/scripts/; temporal_v1_12/scripts/; release_metadata/REPRODUCIBILITY.md</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
@@ -2128,7 +2128,7 @@
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>README_FIRST.md; release_materials/PUBLIC_RELEASE_README.md</t>
+          <t>README.md; release_metadata/REPRODUCIBILITY.md</t>
         </is>
       </c>
       <c r="F8" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Polish submission-facing machine tables
</commit_message>
<xml_diff>
--- a/journal_outputs/machine_readable_tables.xlsx
+++ b/journal_outputs/machine_readable_tables.xlsx
@@ -19,12 +19,12 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="S4_COMPLETE_NULL_CONTROLS" sheetId="10" state="visible" r:id="rId10"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="S5_REFORMS_LOCATION_MATRIX" sheetId="11" state="visible" r:id="rId11"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="S6_DATA_LINEAGE" sheetId="12" state="visible" r:id="rId12"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="S7_NMI_NCS_NONOVERLAP_MATRIX" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="S7_RELATED_PROJECT_BOUNDARY" sheetId="13" state="visible" r:id="rId13"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="S8_DESIGN_AND_FREEZE_AUDIT" sheetId="14" state="visible" r:id="rId14"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="S9_PRIMARY_ENDPOINTS" sheetId="15" state="visible" r:id="rId15"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="S13_TARGET_LEVEL_METRICS" sheetId="16" state="visible" r:id="rId16"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="S14_TARGET_SUPPORT_SENSITIVITY" sheetId="17" state="visible" r:id="rId17"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="S15_NMI_NCS_RECORD_OVERLAP" sheetId="18" state="visible" r:id="rId18"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="S15_RELATED_RECORD_OVERLAP" sheetId="18" state="visible" r:id="rId18"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="S16_INDEPENDENT_SOURCE_RELEASE" sheetId="19" state="visible" r:id="rId19"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="S17_TEMPORAL_MODEL_SPECS" sheetId="20" state="visible" r:id="rId20"/>
   </sheets>
@@ -41,7 +41,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">'S4_COMPLETE_NULL_CONTROLS'!$A$1:$O$19</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="10" hidden="1">'S5_REFORMS_LOCATION_MATRIX'!$A$1:$F$33</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="11" hidden="1">'S6_DATA_LINEAGE'!$A$1:$G$8</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="12" hidden="1">'S7_NMI_NCS_NONOVERLAP_MATRIX'!$A$1:$E$14</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="12" hidden="1">'S7_RELATED_PROJECT_BOUNDARY'!$A$1:$E$14</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="13" hidden="1">'S8_DESIGN_AND_FREEZE_AUDIT'!$A$1:$F$23</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="14" hidden="1">'S9_PRIMARY_ENDPOINTS'!$A$1:$J$17</definedName>
   </definedNames>
@@ -2096,7 +2096,7 @@
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>qc/V1_7_COMPUTE_ENVIRONMENT.txt; qc/V1_7_R_SESSION_INFO.txt; qc/V1_7_FIGURE_BUILD_STATUS.json</t>
+          <t>retrospective_v1_7/qc/V1_7_COMPUTE_ENVIRONMENT.txt; retrospective_v1_7/qc/V1_7_R_SESSION_INFO.txt; qc/V1_7_FIGURE_BUILD_STATUS.json</t>
         </is>
       </c>
       <c r="F7" s="2" t="inlineStr">
@@ -2160,7 +2160,7 @@
       </c>
       <c r="E9" s="2" t="inlineStr">
         <is>
-          <t>scripts/build_v1_7_scientific_upgrade.R; scripts/build_v1_7_figures.R; release_materials/REPRODUCIBILITY_COMMANDS.md</t>
+          <t>retrospective_v1_7/scripts/build_v1_7_scientific_upgrade.R; retrospective_v1_7/scripts/build_v1_7_figures.R; release_materials/REPRODUCIBILITY_COMMANDS.md</t>
         </is>
       </c>
       <c r="F9" s="2" t="inlineStr">
@@ -3255,7 +3255,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E14"/>
+  <dimension ref="A1:D3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="27" customWidth="1" min="1" max="1"/>
@@ -3266,380 +3266,68 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>dimension</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>NMI_v723</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>NCS_v472</t>
-        </is>
-      </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>study_v1_7</t>
-        </is>
-      </c>
-      <c r="E1" s="1" t="inlineStr">
-        <is>
-          <t>boundary_rule</t>
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>related_project</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>scientific_question</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>shared_material</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>boundary_in_this_manuscript</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="inlineStr">
-        <is>
-          <t>central_question</t>
-        </is>
-      </c>
-      <c r="B2" s="2" t="inlineStr">
-        <is>
-          <t>Can released molecular scores retain enough evidence for independent inspection?</t>
-        </is>
-      </c>
-      <c r="C2" s="2" t="inlineStr">
-        <is>
-          <t>Can database release dates be treated as posting times of linked records?</t>
-        </is>
-      </c>
-      <c r="D2" s="2" t="inlineStr">
-        <is>
-          <t>Does source-wide affinity correlation survive hierarchical comparison units, and does it imply within-target ranking or calibrated quantitative transfer?</t>
-        </is>
-      </c>
-      <c r="E2" s="2" t="inlineStr">
-        <is>
-          <t>The present manuscript remains a measurement-validity and external-generalization study.</t>
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>related_molecular_release</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Whether released molecular scores retain enough supporting evidence for independent inspection</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>486 standardized-molecule intersections and 130 five-field Kd payload matches; native activity, assay, document, and measurement-time identifiers were unavailable</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Source reuse only; does not establish exact record overlap, independent replication, or evidence for target-ranking or calibration claims</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="2" t="inlineStr">
-        <is>
-          <t>primary_object</t>
-        </is>
-      </c>
-      <c r="B3" s="2" t="inlineStr">
-        <is>
-          <t>Released score artifacts and evidence bundles</t>
-        </is>
-      </c>
-      <c r="C3" s="2" t="inlineStr">
-        <is>
-          <t>Release records, linked records, and timestamps</t>
-        </is>
-      </c>
-      <c r="D3" s="2" t="inlineStr">
-        <is>
-          <t>External ligand-protein affinity pairs, predictions, errors, intervals, grouping structures, and matched null contrasts</t>
-        </is>
-      </c>
-      <c r="E3" s="2" t="inlineStr">
-        <is>
-          <t>Release artifacts and evidence clocks do not enter the outcome model.</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="2" t="inlineStr">
-        <is>
-          <t>unit_of_analysis</t>
-        </is>
-      </c>
-      <c r="B4" s="2" t="inlineStr">
-        <is>
-          <t>Released output or audit question</t>
-        </is>
-      </c>
-      <c r="C4" s="2" t="inlineStr">
-        <is>
-          <t>Release-record-document linkage</t>
-        </is>
-      </c>
-      <c r="D4" s="2" t="inlineStr">
-        <is>
-          <t>Affinity pair with connected-document, scaffold, exact-protein, and protein-cluster dependence</t>
-        </is>
-      </c>
-      <c r="E4" s="2" t="inlineStr">
-        <is>
-          <t>Statistical inference uses predictive and hierarchical molecular units only.</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="2" t="inlineStr">
-        <is>
-          <t>core_outcome</t>
-        </is>
-      </c>
-      <c r="B5" s="2" t="inlineStr">
-        <is>
-          <t>Evidence retention and answer identifiability</t>
-        </is>
-      </c>
-      <c r="C5" s="2" t="inlineStr">
-        <is>
-          <t>Timestamp mismatch and chronology semantics</t>
-        </is>
-      </c>
-      <c r="D5" s="2" t="inlineStr">
-        <is>
-          <t>Source-wide and within-context rank, point accuracy against fixed references, calibration, coverage, composition sensitivity, and permutation contrasts</t>
-        </is>
-      </c>
-      <c r="E5" s="2" t="inlineStr">
-        <is>
-          <t>Prediction failure is not reframed as governance or chronology.</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="2" t="inlineStr">
-        <is>
-          <t>main_exposure</t>
-        </is>
-      </c>
-      <c r="B6" s="2" t="inlineStr">
-        <is>
-          <t>Evidence retained by a release contract</t>
-        </is>
-      </c>
-      <c r="C6" s="2" t="inlineStr">
-        <is>
-          <t>Choice of timestamp or evidence clock</t>
-        </is>
-      </c>
-      <c r="D6" s="2" t="inlineStr">
-        <is>
-          <t>External source, cold-start category, comparison unit, model specification, assay-context alignment, and geometry alignment</t>
-        </is>
-      </c>
-      <c r="E6" s="2" t="inlineStr">
-        <is>
-          <t>No release-contract or timestamp exposure is reused.</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="2" t="inlineStr">
-        <is>
-          <t>study_design</t>
-        </is>
-      </c>
-      <c r="B7" s="2" t="inlineStr">
-        <is>
-          <t>Released-output reconstruction</t>
-        </is>
-      </c>
-      <c r="C7" s="2" t="inlineStr">
-        <is>
-          <t>Cross-record chronology analysis</t>
-        </is>
-      </c>
-      <c r="D7" s="2" t="inlineStr">
-        <is>
-          <t>Frozen external predictions plus retrospective hierarchical decomposition, crossed-dependence inference, influence diagnostics, and outcome-unexposed, structure-adapted temporal validation</t>
-        </is>
-      </c>
-      <c r="E7" s="2" t="inlineStr">
-        <is>
-          <t>Shared hashes and infrastructure appear only as provenance.</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="2" t="inlineStr">
-        <is>
-          <t>headline_claim</t>
-        </is>
-      </c>
-      <c r="B8" s="2" t="inlineStr">
-        <is>
-          <t>Scores can outlive the evidence needed to inspect them</t>
-        </is>
-      </c>
-      <c r="C8" s="2" t="inlineStr">
-        <is>
-          <t>Release time need not equal linked-record posting time</t>
-        </is>
-      </c>
-      <c r="D8" s="2" t="inlineStr">
-        <is>
-          <t>Reproducible source-wide rank association can be dominated by between-document and between-target composition and need not establish within-target ligand ranking or calibrated transfer</t>
-        </is>
-      </c>
-      <c r="E8" s="2" t="inlineStr">
-        <is>
-          <t>No headline or conceptual framing is shared.</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="2" t="inlineStr">
-        <is>
-          <t>main_figures</t>
-        </is>
-      </c>
-      <c r="B9" s="2" t="inlineStr">
-        <is>
-          <t>Release artifacts and evidence preservation</t>
-        </is>
-      </c>
-      <c r="C9" s="2" t="inlineStr">
-        <is>
-          <t>Timestamp mismatch and evidence-clock diagrams</t>
-        </is>
-      </c>
-      <c r="D9" s="2" t="inlineStr">
-        <is>
-          <t>Hierarchical support, rank inference, covariance decomposition, composition sensitivity, conditional uncertainty, feature-null heterogeneity, and claim boundary</t>
-        </is>
-      </c>
-      <c r="E9" s="2" t="inlineStr">
-        <is>
-          <t>No governance or timestamp panel appears in Figs. 1-6.</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="2" t="inlineStr">
-        <is>
-          <t>reserved_language</t>
-        </is>
-      </c>
-      <c r="B10" s="2" t="inlineStr">
-        <is>
-          <t>release contract; evidence bundle; non-identifiability</t>
-        </is>
-      </c>
-      <c r="C10" s="2" t="inlineStr">
-        <is>
-          <t>release time; posting time; evidence clock</t>
-        </is>
-      </c>
-      <c r="D10" s="2" t="inlineStr">
-        <is>
-          <t>comparison unit; source shift; within-context rank; clustered inference; poststratification; conditional coverage</t>
-        </is>
-      </c>
-      <c r="E10" s="2" t="inlineStr">
-        <is>
-          <t>NMI/NCS reserved terms are excluded except when identifying related manuscripts.</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="2" t="inlineStr">
-        <is>
-          <t>allowed_bridge</t>
-        </is>
-      </c>
-      <c r="B11" s="2" t="inlineStr">
-        <is>
-          <t>Dataset provenance only</t>
-        </is>
-      </c>
-      <c r="C11" s="2" t="inlineStr">
-        <is>
-          <t>Dataset provenance only</t>
-        </is>
-      </c>
-      <c r="D11" s="2" t="inlineStr">
-        <is>
-          <t>Frozen hashes, database identifiers, overlap counts, rights restrictions, and related-manuscript disclosure</t>
-        </is>
-      </c>
-      <c r="E11" s="2" t="inlineStr">
-        <is>
-          <t>A provenance statement cannot become a conceptual contribution.</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="2" t="inlineStr">
-        <is>
-          <t>disease_or_candidate_case</t>
-        </is>
-      </c>
-      <c r="B12" s="2" t="inlineStr">
-        <is>
-          <t>not required</t>
-        </is>
-      </c>
-      <c r="C12" s="2" t="inlineStr">
-        <is>
-          <t>not required</t>
-        </is>
-      </c>
-      <c r="D12" s="2" t="inlineStr">
-        <is>
-          <t>No DMD/HDAC6, disease mechanism, ADMET, target nomination, or therapeutic candidate validation</t>
-        </is>
-      </c>
-      <c r="E12" s="2" t="inlineStr">
-        <is>
-          <t>Disease and therapeutic branches cannot be reused as evidence.</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="2" t="inlineStr">
-        <is>
-          <t>publication_identity</t>
-        </is>
-      </c>
-      <c r="B13" s="2" t="inlineStr">
-        <is>
-          <t>release-auditability manuscript</t>
-        </is>
-      </c>
-      <c r="C13" s="2" t="inlineStr">
-        <is>
-          <t>evidence-chronology manuscript</t>
-        </is>
-      </c>
-      <c r="D13" s="2" t="inlineStr">
-        <is>
-          <t>hierarchical external-validation and benchmark-measurement manuscript</t>
-        </is>
-      </c>
-      <c r="E13" s="2" t="inlineStr">
-        <is>
-          <t>Title, abstract, estimands, figures, and conclusions remain independently identifiable.</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="2" t="inlineStr">
-        <is>
-          <t>overlap_audit_action</t>
-        </is>
-      </c>
-      <c r="B14" s="2" t="inlineStr">
-        <is>
-          <t>Disclose as related manuscript</t>
-        </is>
-      </c>
-      <c r="C14" s="2" t="inlineStr">
-        <is>
-          <t>Disclose as related manuscript</t>
-        </is>
-      </c>
-      <c r="D14" s="2" t="inlineStr">
-        <is>
-          <t>Upload both manuscripts if submitted or in review and provide this matrix to the corresponding author</t>
-        </is>
-      </c>
-      <c r="E14" s="2" t="inlineStr">
-        <is>
-          <t>Editors decide publication overlap; this matrix does not replace disclosure.</t>
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>related_forward_activity_release</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>How database and document timestamps relate to the chronology of linked activity records</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>5,215 native ChEMBL activity IDs overlap the raw ChEMBL37 snapshot, including 256 in curated external pairs; separately reviewed full-text ledger has zero exact-ID matches</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Shared source identifiers only; no claim about evidence emergence, database posting, or relation-formation chronology</t>
         </is>
       </c>
     </row>

</xml_diff>